<commit_message>
Fix industry classification for remaining QNC silo tasks
Ensure C00008036 conveyor tasks are tagged as industrial in summary sheets.

Co-authored-by: liborvybral-collab <liborvybral-collab@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/presentations/management-biweekly/2026/2026-07-23-方案报价任务业务员明细.xlsx
+++ b/docs/presentations/management-biweekly/2026/2026-07-23-方案报价任务业务员明细.xlsx
@@ -518,7 +518,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7">
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11">
@@ -1944,7 +1944,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1976,51 +1976,35 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>工业</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>91</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>157</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>工业</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>92</v>
+      </c>
+      <c r="C2" t="n">
+        <v>67</v>
+      </c>
+      <c r="D2" t="n">
+        <v>159</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>粮食</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" t="n">
         <v>56</v>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" t="n">
         <v>39</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" t="n">
         <v>95</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -5670,7 +5654,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -14061,7 +14045,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>工业</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">

</xml_diff>